<commit_message>
Add MSG91 SMS and WhatsApp automation feature to backlog; update V1 launch checklist and add dev deployment checklist
</commit_message>
<xml_diff>
--- a/docs/customer-frontend-qa-checklist-local-env.xlsx
+++ b/docs/customer-frontend-qa-checklist-local-env.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ayanc\OneDrive\Desktop\cabbo-frontends\cabbo-customer-frontend\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C2F513F-62B2-4B05-9DBC-9DED6A96B019}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1C656D1-2AE6-41CF-AF3E-E08E26A4DCA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -701,9 +701,6 @@
   </si>
   <si>
     <t>Customer A (Ayan)</t>
-  </si>
-  <si>
-    <t>Customer B (Oyendrila</t>
   </si>
   <si>
     <t>Successful login/onboarding with OTP</t>
@@ -835,6 +832,9 @@
       </rPr>
       <t>" which clearly is an email validation error during creating the payment order. Hence the screen shows a Error Boundary generic screen, but funny part is when we retry on the generic error page or refresh the page - the error does not happen any more and initiates the booking successfully.</t>
     </r>
+  </si>
+  <si>
+    <t>Customer B (Oyendrila)</t>
   </si>
 </sst>
 </file>
@@ -1476,7 +1476,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1633,16 +1633,16 @@
         <v>9831305667</v>
       </c>
       <c r="F2" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="G2" s="14" t="s">
         <v>226</v>
-      </c>
-      <c r="G2" s="14" t="s">
-        <v>227</v>
       </c>
       <c r="H2" s="2"/>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" s="8" t="s">
-        <v>225</v>
+        <v>260</v>
       </c>
       <c r="B3" s="8" t="s">
         <v>18</v>
@@ -1657,10 +1657,10 @@
         <v>8017084241</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="H3" s="2"/>
     </row>
@@ -1759,10 +1759,10 @@
         <v>38</v>
       </c>
       <c r="G2" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I2" s="9">
         <v>46208</v>
@@ -1792,10 +1792,10 @@
         <v>42</v>
       </c>
       <c r="G3" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I3" s="9">
         <v>46208</v>
@@ -1825,10 +1825,10 @@
         <v>48</v>
       </c>
       <c r="G4" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I4" s="9">
         <v>46208</v>
@@ -1858,10 +1858,10 @@
         <v>50</v>
       </c>
       <c r="G5" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I5" s="9">
         <v>46208</v>
@@ -1891,10 +1891,10 @@
         <v>52</v>
       </c>
       <c r="G6" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I6" s="9">
         <v>46208</v>
@@ -1924,10 +1924,10 @@
         <v>54</v>
       </c>
       <c r="G7" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I7" s="9">
         <v>46208</v>
@@ -1957,10 +1957,10 @@
         <v>58</v>
       </c>
       <c r="G8" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I8" s="9">
         <v>46208</v>
@@ -1990,10 +1990,10 @@
         <v>61</v>
       </c>
       <c r="G9" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I9" s="9">
         <v>46208</v>
@@ -2023,10 +2023,10 @@
         <v>64</v>
       </c>
       <c r="G10" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I10" s="9">
         <v>46208</v>
@@ -2056,10 +2056,10 @@
         <v>67</v>
       </c>
       <c r="G11" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I11" s="9">
         <v>46208</v>
@@ -2089,10 +2089,10 @@
         <v>70</v>
       </c>
       <c r="G12" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I12" s="9">
         <v>46208</v>
@@ -2122,10 +2122,10 @@
         <v>74</v>
       </c>
       <c r="G13" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I13" s="9">
         <v>46208</v>
@@ -2155,10 +2155,10 @@
         <v>77</v>
       </c>
       <c r="G14" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I14" s="9">
         <v>46208</v>
@@ -2188,10 +2188,10 @@
         <v>81</v>
       </c>
       <c r="G15" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I15" s="9">
         <v>46208</v>
@@ -2221,10 +2221,10 @@
         <v>84</v>
       </c>
       <c r="G16" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I16" s="9">
         <v>46208</v>
@@ -2254,10 +2254,10 @@
         <v>87</v>
       </c>
       <c r="G17" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H17" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I17" s="9">
         <v>46208</v>
@@ -2287,10 +2287,10 @@
         <v>91</v>
       </c>
       <c r="G18" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H18" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I18" s="9">
         <v>46208</v>
@@ -2320,10 +2320,10 @@
         <v>94</v>
       </c>
       <c r="G19" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H19" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I19" s="9">
         <v>46208</v>
@@ -2353,10 +2353,10 @@
         <v>97</v>
       </c>
       <c r="G20" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H20" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I20" s="9">
         <v>46208</v>
@@ -2386,10 +2386,10 @@
         <v>100</v>
       </c>
       <c r="G21" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H21" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I21" s="9">
         <v>46208</v>
@@ -2419,10 +2419,10 @@
         <v>103</v>
       </c>
       <c r="G22" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H22" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I22" s="9">
         <v>46208</v>
@@ -2452,10 +2452,10 @@
         <v>107</v>
       </c>
       <c r="G23" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H23" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I23" s="9">
         <v>46208</v>
@@ -2485,10 +2485,10 @@
         <v>110</v>
       </c>
       <c r="G24" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H24" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I24" s="9">
         <v>46208</v>
@@ -2518,10 +2518,10 @@
         <v>114</v>
       </c>
       <c r="G25" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H25" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I25" s="9">
         <v>46208</v>
@@ -2551,10 +2551,10 @@
         <v>117</v>
       </c>
       <c r="G26" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H26" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I26" s="9">
         <v>46208</v>
@@ -2584,10 +2584,10 @@
         <v>120</v>
       </c>
       <c r="G27" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H27" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I27" s="9">
         <v>46208</v>
@@ -2617,10 +2617,10 @@
         <v>125</v>
       </c>
       <c r="G28" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H28" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I28" s="9">
         <v>46208</v>
@@ -2653,7 +2653,7 @@
         <v>39</v>
       </c>
       <c r="H29" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I29" s="9"/>
       <c r="J29" s="8"/>
@@ -2684,7 +2684,7 @@
         <v>39</v>
       </c>
       <c r="H30" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I30" s="9"/>
       <c r="J30" s="8"/>
@@ -2712,10 +2712,10 @@
         <v>134</v>
       </c>
       <c r="G31" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H31" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I31" s="9">
         <v>46208</v>
@@ -2748,7 +2748,7 @@
         <v>39</v>
       </c>
       <c r="H32" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I32" s="8"/>
       <c r="J32" s="8"/>
@@ -2779,7 +2779,7 @@
         <v>39</v>
       </c>
       <c r="H33" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I33" s="8"/>
       <c r="J33" s="8"/>
@@ -2810,7 +2810,7 @@
         <v>39</v>
       </c>
       <c r="H34" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I34" s="8"/>
       <c r="J34" s="8"/>
@@ -2838,10 +2838,10 @@
         <v>146</v>
       </c>
       <c r="G35" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H35" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I35" s="9">
         <v>46208</v>
@@ -2871,10 +2871,10 @@
         <v>151</v>
       </c>
       <c r="G36" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H36" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I36" s="9">
         <v>46208</v>
@@ -2904,10 +2904,10 @@
         <v>155</v>
       </c>
       <c r="G37" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H37" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I37" s="9">
         <v>46208</v>
@@ -2934,13 +2934,13 @@
         <v>157</v>
       </c>
       <c r="F38" s="8" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="G38" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H38" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I38" s="9">
         <v>46208</v>
@@ -2970,10 +2970,10 @@
         <v>162</v>
       </c>
       <c r="G39" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H39" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I39" s="9">
         <v>46208</v>
@@ -3000,13 +3000,13 @@
         <v>165</v>
       </c>
       <c r="F40" s="8" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="G40" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H40" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I40" s="9">
         <v>46208</v>
@@ -3036,10 +3036,10 @@
         <v>171</v>
       </c>
       <c r="G41" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H41" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I41" s="9">
         <v>46208</v>
@@ -3069,10 +3069,10 @@
         <v>174</v>
       </c>
       <c r="G42" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H42" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I42" s="9">
         <v>46208</v>
@@ -3102,10 +3102,10 @@
         <v>179</v>
       </c>
       <c r="G43" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H43" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I43" s="9">
         <v>46208</v>
@@ -3135,10 +3135,10 @@
         <v>182</v>
       </c>
       <c r="G44" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H44" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I44" s="9">
         <v>46208</v>
@@ -3168,10 +3168,10 @@
         <v>185</v>
       </c>
       <c r="G45" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H45" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I45" s="9">
         <v>46208</v>
@@ -3201,10 +3201,10 @@
         <v>190</v>
       </c>
       <c r="G46" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H46" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I46" s="9">
         <v>46208</v>
@@ -3234,10 +3234,10 @@
         <v>192</v>
       </c>
       <c r="G47" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H47" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I47" s="9">
         <v>46208</v>
@@ -3267,10 +3267,10 @@
         <v>194</v>
       </c>
       <c r="G48" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H48" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I48" s="9">
         <v>46208</v>
@@ -3300,10 +3300,10 @@
         <v>196</v>
       </c>
       <c r="G49" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H49" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I49" s="9">
         <v>46208</v>
@@ -3333,10 +3333,10 @@
         <v>198</v>
       </c>
       <c r="G50" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H50" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I50" s="9">
         <v>46208</v>
@@ -3366,10 +3366,10 @@
         <v>203</v>
       </c>
       <c r="G51" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H51" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I51" s="9">
         <v>46208</v>
@@ -3399,10 +3399,10 @@
         <v>207</v>
       </c>
       <c r="G52" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H52" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I52" s="9">
         <v>46208</v>
@@ -3432,10 +3432,10 @@
         <v>212</v>
       </c>
       <c r="G53" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H53" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I53" s="9">
         <v>46208</v>
@@ -3465,10 +3465,10 @@
         <v>212</v>
       </c>
       <c r="G54" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H54" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I54" s="9">
         <v>46208</v>
@@ -3486,7 +3486,7 @@
         <v>209</v>
       </c>
       <c r="C55" s="8" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="D55" s="8" t="s">
         <v>46</v>
@@ -3498,10 +3498,10 @@
         <v>212</v>
       </c>
       <c r="G55" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H55" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I55" s="9">
         <v>46208</v>
@@ -3531,10 +3531,10 @@
         <v>212</v>
       </c>
       <c r="G56" s="15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H56" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I56" s="9">
         <v>46208</v>
@@ -3567,7 +3567,7 @@
         <v>4</v>
       </c>
       <c r="H57" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I57" s="8"/>
       <c r="J57" s="8"/>
@@ -3591,7 +3591,7 @@
     </row>
     <row r="70" spans="13:13">
       <c r="M70" s="4" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="71" spans="13:13">
@@ -3601,12 +3601,12 @@
     </row>
     <row r="72" spans="13:13">
       <c r="M72" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="73" spans="13:13">
       <c r="M73" s="3" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="74" spans="13:13">
@@ -3661,7 +3661,7 @@
         <v>220</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="E1" s="7" t="s">
         <v>221</v>
@@ -3687,25 +3687,25 @@
         <v>33</v>
       </c>
       <c r="D2" s="18" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E2" s="18" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F2" s="18" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G2" s="18" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="H2" s="18" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="I2" s="2"/>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" s="18" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B3" s="19">
         <v>46208</v>
@@ -3714,25 +3714,25 @@
         <v>44</v>
       </c>
       <c r="D3" s="18" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E3" s="18" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G3" s="18" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="H3" s="18" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="I3" s="2"/>
     </row>
     <row r="4" spans="1:9" s="12" customFormat="1" ht="159.5">
       <c r="A4" s="20" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B4" s="16">
         <v>46208</v>
@@ -3741,25 +3741,25 @@
         <v>108</v>
       </c>
       <c r="D4" s="20" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E4" s="20" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="F4" s="20" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G4" s="20" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="H4" s="21" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="I4" s="11"/>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" s="18" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B5" s="19">
         <v>46208</v>
@@ -3768,100 +3768,100 @@
         <v>118</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G5" s="18" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="H5" s="18" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="I5" s="2"/>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" s="18" t="s">
+        <v>246</v>
+      </c>
+      <c r="B6" s="19">
+        <v>46208</v>
+      </c>
+      <c r="C6" s="18" t="s">
+        <v>248</v>
+      </c>
+      <c r="D6" s="18" t="s">
+        <v>249</v>
+      </c>
+      <c r="E6" s="18" t="s">
+        <v>240</v>
+      </c>
+      <c r="F6" s="18" t="s">
+        <v>258</v>
+      </c>
+      <c r="G6" s="18" t="s">
+        <v>228</v>
+      </c>
+      <c r="H6" s="18" t="s">
         <v>247</v>
-      </c>
-      <c r="B6" s="19">
-        <v>46208</v>
-      </c>
-      <c r="C6" s="18" t="s">
-        <v>249</v>
-      </c>
-      <c r="D6" s="18" t="s">
-        <v>250</v>
-      </c>
-      <c r="E6" s="18" t="s">
-        <v>241</v>
-      </c>
-      <c r="F6" s="18" t="s">
-        <v>259</v>
-      </c>
-      <c r="G6" s="18" t="s">
-        <v>229</v>
-      </c>
-      <c r="H6" s="18" t="s">
-        <v>248</v>
       </c>
       <c r="I6" s="2"/>
     </row>
     <row r="7" spans="1:9">
       <c r="A7" s="18" t="s">
+        <v>250</v>
+      </c>
+      <c r="B7" s="19">
+        <v>46208</v>
+      </c>
+      <c r="C7" s="18" t="s">
         <v>251</v>
       </c>
-      <c r="B7" s="19">
-        <v>46208</v>
-      </c>
-      <c r="C7" s="18" t="s">
+      <c r="D7" s="18" t="s">
         <v>252</v>
       </c>
-      <c r="D7" s="18" t="s">
-        <v>253</v>
-      </c>
       <c r="E7" s="18" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G7" s="18" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="H7" s="18" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="I7" s="2"/>
     </row>
     <row r="8" spans="1:9" s="17" customFormat="1" ht="290">
       <c r="A8" s="20" t="s">
+        <v>255</v>
+      </c>
+      <c r="B8" s="16">
+        <v>46208</v>
+      </c>
+      <c r="C8" s="23" t="s">
         <v>256</v>
       </c>
-      <c r="B8" s="16">
-        <v>46208</v>
-      </c>
-      <c r="C8" s="23" t="s">
+      <c r="D8" s="23" t="s">
         <v>257</v>
       </c>
-      <c r="D8" s="23" t="s">
+      <c r="E8" s="23" t="s">
+        <v>240</v>
+      </c>
+      <c r="F8" s="23" t="s">
         <v>258</v>
       </c>
-      <c r="E8" s="23" t="s">
-        <v>241</v>
-      </c>
-      <c r="F8" s="23" t="s">
+      <c r="G8" s="23" t="s">
+        <v>228</v>
+      </c>
+      <c r="H8" s="24" t="s">
         <v>259</v>
-      </c>
-      <c r="G8" s="23" t="s">
-        <v>229</v>
-      </c>
-      <c r="H8" s="24" t="s">
-        <v>260</v>
       </c>
       <c r="I8" s="22"/>
     </row>

</xml_diff>

<commit_message>
Update deployment documentation and improve login handling in LegalPage and VerifyEmailPage components; enhance UI in Login component
</commit_message>
<xml_diff>
--- a/docs/customer-frontend-qa-checklist-local-env.xlsx
+++ b/docs/customer-frontend-qa-checklist-local-env.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ayanc\OneDrive\Desktop\cabbo-frontends\cabbo-customer-frontend\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1C656D1-2AE6-41CF-AF3E-E08E26A4DCA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F7DA8BB-8201-4987-A2D3-10344B5C3755}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="554" uniqueCount="261">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="559" uniqueCount="262">
   <si>
     <t>Generated for local QA run</t>
   </si>
@@ -835,6 +835,9 @@
   </si>
   <si>
     <t>Customer B (Oyendrila)</t>
+  </si>
+  <si>
+    <t>Will do once I complete admin panel - so I can enough data to perform this step</t>
   </si>
 </sst>
 </file>
@@ -1683,6 +1686,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:M75"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
@@ -1739,7 +1743,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:13">
+    <row r="2" spans="1:13" hidden="1">
       <c r="A2" s="8" t="s">
         <v>33</v>
       </c>
@@ -1772,7 +1776,7 @@
       <c r="L2" s="8"/>
       <c r="M2" s="2"/>
     </row>
-    <row r="3" spans="1:13">
+    <row r="3" spans="1:13" hidden="1">
       <c r="A3" s="8" t="s">
         <v>33</v>
       </c>
@@ -1805,7 +1809,7 @@
       <c r="L3" s="8"/>
       <c r="M3" s="2"/>
     </row>
-    <row r="4" spans="1:13">
+    <row r="4" spans="1:13" hidden="1">
       <c r="A4" s="8" t="s">
         <v>43</v>
       </c>
@@ -1838,7 +1842,7 @@
       <c r="L4" s="8"/>
       <c r="M4" s="2"/>
     </row>
-    <row r="5" spans="1:13">
+    <row r="5" spans="1:13" hidden="1">
       <c r="A5" s="8" t="s">
         <v>43</v>
       </c>
@@ -1871,7 +1875,7 @@
       <c r="L5" s="8"/>
       <c r="M5" s="2"/>
     </row>
-    <row r="6" spans="1:13">
+    <row r="6" spans="1:13" hidden="1">
       <c r="A6" s="8" t="s">
         <v>43</v>
       </c>
@@ -1904,7 +1908,7 @@
       <c r="L6" s="8"/>
       <c r="M6" s="2"/>
     </row>
-    <row r="7" spans="1:13">
+    <row r="7" spans="1:13" hidden="1">
       <c r="A7" s="8" t="s">
         <v>43</v>
       </c>
@@ -1937,7 +1941,7 @@
       <c r="L7" s="8"/>
       <c r="M7" s="2"/>
     </row>
-    <row r="8" spans="1:13">
+    <row r="8" spans="1:13" hidden="1">
       <c r="A8" s="8" t="s">
         <v>43</v>
       </c>
@@ -1970,7 +1974,7 @@
       <c r="L8" s="8"/>
       <c r="M8" s="2"/>
     </row>
-    <row r="9" spans="1:13">
+    <row r="9" spans="1:13" hidden="1">
       <c r="A9" s="8" t="s">
         <v>43</v>
       </c>
@@ -2003,7 +2007,7 @@
       <c r="L9" s="8"/>
       <c r="M9" s="2"/>
     </row>
-    <row r="10" spans="1:13">
+    <row r="10" spans="1:13" hidden="1">
       <c r="A10" s="8" t="s">
         <v>43</v>
       </c>
@@ -2036,7 +2040,7 @@
       <c r="L10" s="8"/>
       <c r="M10" s="2"/>
     </row>
-    <row r="11" spans="1:13">
+    <row r="11" spans="1:13" hidden="1">
       <c r="A11" s="8" t="s">
         <v>43</v>
       </c>
@@ -2069,7 +2073,7 @@
       <c r="L11" s="8"/>
       <c r="M11" s="2"/>
     </row>
-    <row r="12" spans="1:13">
+    <row r="12" spans="1:13" hidden="1">
       <c r="A12" s="8" t="s">
         <v>43</v>
       </c>
@@ -2102,7 +2106,7 @@
       <c r="L12" s="8"/>
       <c r="M12" s="2"/>
     </row>
-    <row r="13" spans="1:13">
+    <row r="13" spans="1:13" hidden="1">
       <c r="A13" s="8" t="s">
         <v>71</v>
       </c>
@@ -2135,7 +2139,7 @@
       <c r="L13" s="8"/>
       <c r="M13" s="2"/>
     </row>
-    <row r="14" spans="1:13">
+    <row r="14" spans="1:13" hidden="1">
       <c r="A14" s="8" t="s">
         <v>71</v>
       </c>
@@ -2168,7 +2172,7 @@
       <c r="L14" s="8"/>
       <c r="M14" s="2"/>
     </row>
-    <row r="15" spans="1:13">
+    <row r="15" spans="1:13" hidden="1">
       <c r="A15" s="8" t="s">
         <v>78</v>
       </c>
@@ -2201,7 +2205,7 @@
       <c r="L15" s="8"/>
       <c r="M15" s="2"/>
     </row>
-    <row r="16" spans="1:13">
+    <row r="16" spans="1:13" hidden="1">
       <c r="A16" s="8" t="s">
         <v>78</v>
       </c>
@@ -2234,7 +2238,7 @@
       <c r="L16" s="8"/>
       <c r="M16" s="2"/>
     </row>
-    <row r="17" spans="1:13">
+    <row r="17" spans="1:13" hidden="1">
       <c r="A17" s="8" t="s">
         <v>78</v>
       </c>
@@ -2267,7 +2271,7 @@
       <c r="L17" s="8"/>
       <c r="M17" s="2"/>
     </row>
-    <row r="18" spans="1:13">
+    <row r="18" spans="1:13" hidden="1">
       <c r="A18" s="8" t="s">
         <v>88</v>
       </c>
@@ -2300,7 +2304,7 @@
       <c r="L18" s="8"/>
       <c r="M18" s="2"/>
     </row>
-    <row r="19" spans="1:13">
+    <row r="19" spans="1:13" hidden="1">
       <c r="A19" s="8" t="s">
         <v>88</v>
       </c>
@@ -2333,7 +2337,7 @@
       <c r="L19" s="8"/>
       <c r="M19" s="2"/>
     </row>
-    <row r="20" spans="1:13">
+    <row r="20" spans="1:13" hidden="1">
       <c r="A20" s="8" t="s">
         <v>88</v>
       </c>
@@ -2366,7 +2370,7 @@
       <c r="L20" s="8"/>
       <c r="M20" s="2"/>
     </row>
-    <row r="21" spans="1:13">
+    <row r="21" spans="1:13" hidden="1">
       <c r="A21" s="8" t="s">
         <v>88</v>
       </c>
@@ -2399,7 +2403,7 @@
       <c r="L21" s="8"/>
       <c r="M21" s="2"/>
     </row>
-    <row r="22" spans="1:13">
+    <row r="22" spans="1:13" hidden="1">
       <c r="A22" s="8" t="s">
         <v>88</v>
       </c>
@@ -2432,7 +2436,7 @@
       <c r="L22" s="8"/>
       <c r="M22" s="2"/>
     </row>
-    <row r="23" spans="1:13">
+    <row r="23" spans="1:13" hidden="1">
       <c r="A23" s="8" t="s">
         <v>104</v>
       </c>
@@ -2465,7 +2469,7 @@
       <c r="L23" s="8"/>
       <c r="M23" s="2"/>
     </row>
-    <row r="24" spans="1:13">
+    <row r="24" spans="1:13" hidden="1">
       <c r="A24" s="8" t="s">
         <v>104</v>
       </c>
@@ -2498,7 +2502,7 @@
       <c r="L24" s="10"/>
       <c r="M24" s="2"/>
     </row>
-    <row r="25" spans="1:13">
+    <row r="25" spans="1:13" hidden="1">
       <c r="A25" s="8" t="s">
         <v>111</v>
       </c>
@@ -2531,7 +2535,7 @@
       <c r="L25" s="8"/>
       <c r="M25" s="2"/>
     </row>
-    <row r="26" spans="1:13">
+    <row r="26" spans="1:13" hidden="1">
       <c r="A26" s="8" t="s">
         <v>111</v>
       </c>
@@ -2564,7 +2568,7 @@
       <c r="L26" s="8"/>
       <c r="M26" s="2"/>
     </row>
-    <row r="27" spans="1:13">
+    <row r="27" spans="1:13" hidden="1">
       <c r="A27" s="8" t="s">
         <v>111</v>
       </c>
@@ -2597,7 +2601,7 @@
       <c r="L27" s="8"/>
       <c r="M27" s="2"/>
     </row>
-    <row r="28" spans="1:13">
+    <row r="28" spans="1:13" hidden="1">
       <c r="A28" s="8" t="s">
         <v>121</v>
       </c>
@@ -2658,7 +2662,9 @@
       <c r="I29" s="9"/>
       <c r="J29" s="8"/>
       <c r="K29" s="8"/>
-      <c r="L29" s="8"/>
+      <c r="L29" s="8" t="s">
+        <v>261</v>
+      </c>
       <c r="M29" s="2"/>
     </row>
     <row r="30" spans="1:13">
@@ -2689,10 +2695,12 @@
       <c r="I30" s="9"/>
       <c r="J30" s="8"/>
       <c r="K30" s="8"/>
-      <c r="L30" s="8"/>
+      <c r="L30" s="8" t="s">
+        <v>261</v>
+      </c>
       <c r="M30" s="2"/>
     </row>
-    <row r="31" spans="1:13">
+    <row r="31" spans="1:13" hidden="1">
       <c r="A31" s="8" t="s">
         <v>121</v>
       </c>
@@ -2753,7 +2761,9 @@
       <c r="I32" s="8"/>
       <c r="J32" s="8"/>
       <c r="K32" s="8"/>
-      <c r="L32" s="8"/>
+      <c r="L32" s="8" t="s">
+        <v>261</v>
+      </c>
       <c r="M32" s="2"/>
     </row>
     <row r="33" spans="1:13">
@@ -2784,7 +2794,9 @@
       <c r="I33" s="8"/>
       <c r="J33" s="8"/>
       <c r="K33" s="8"/>
-      <c r="L33" s="8"/>
+      <c r="L33" s="8" t="s">
+        <v>261</v>
+      </c>
       <c r="M33" s="2"/>
     </row>
     <row r="34" spans="1:13">
@@ -2815,10 +2827,12 @@
       <c r="I34" s="8"/>
       <c r="J34" s="8"/>
       <c r="K34" s="8"/>
-      <c r="L34" s="8"/>
+      <c r="L34" s="8" t="s">
+        <v>261</v>
+      </c>
       <c r="M34" s="2"/>
     </row>
-    <row r="35" spans="1:13">
+    <row r="35" spans="1:13" hidden="1">
       <c r="A35" s="8" t="s">
         <v>141</v>
       </c>
@@ -2851,7 +2865,7 @@
       <c r="L35" s="8"/>
       <c r="M35" s="2"/>
     </row>
-    <row r="36" spans="1:13">
+    <row r="36" spans="1:13" hidden="1">
       <c r="A36" s="8" t="s">
         <v>147</v>
       </c>
@@ -2884,7 +2898,7 @@
       <c r="L36" s="8"/>
       <c r="M36" s="2"/>
     </row>
-    <row r="37" spans="1:13">
+    <row r="37" spans="1:13" hidden="1">
       <c r="A37" s="8" t="s">
         <v>147</v>
       </c>
@@ -2917,7 +2931,7 @@
       <c r="L37" s="8"/>
       <c r="M37" s="2"/>
     </row>
-    <row r="38" spans="1:13">
+    <row r="38" spans="1:13" hidden="1">
       <c r="A38" s="8" t="s">
         <v>147</v>
       </c>
@@ -2950,7 +2964,7 @@
       <c r="L38" s="8"/>
       <c r="M38" s="2"/>
     </row>
-    <row r="39" spans="1:13">
+    <row r="39" spans="1:13" hidden="1">
       <c r="A39" s="8" t="s">
         <v>158</v>
       </c>
@@ -2983,7 +2997,7 @@
       <c r="L39" s="8"/>
       <c r="M39" s="2"/>
     </row>
-    <row r="40" spans="1:13">
+    <row r="40" spans="1:13" hidden="1">
       <c r="A40" s="8" t="s">
         <v>158</v>
       </c>
@@ -3016,7 +3030,7 @@
       <c r="L40" s="8"/>
       <c r="M40" s="2"/>
     </row>
-    <row r="41" spans="1:13">
+    <row r="41" spans="1:13" hidden="1">
       <c r="A41" s="8" t="s">
         <v>166</v>
       </c>
@@ -3049,7 +3063,7 @@
       <c r="L41" s="8"/>
       <c r="M41" s="2"/>
     </row>
-    <row r="42" spans="1:13">
+    <row r="42" spans="1:13" hidden="1">
       <c r="A42" s="8" t="s">
         <v>166</v>
       </c>
@@ -3082,7 +3096,7 @@
       <c r="L42" s="8"/>
       <c r="M42" s="2"/>
     </row>
-    <row r="43" spans="1:13">
+    <row r="43" spans="1:13" hidden="1">
       <c r="A43" s="8" t="s">
         <v>166</v>
       </c>
@@ -3115,7 +3129,7 @@
       <c r="L43" s="8"/>
       <c r="M43" s="2"/>
     </row>
-    <row r="44" spans="1:13">
+    <row r="44" spans="1:13" hidden="1">
       <c r="A44" s="8" t="s">
         <v>166</v>
       </c>
@@ -3148,7 +3162,7 @@
       <c r="L44" s="8"/>
       <c r="M44" s="2"/>
     </row>
-    <row r="45" spans="1:13">
+    <row r="45" spans="1:13" hidden="1">
       <c r="A45" s="8" t="s">
         <v>166</v>
       </c>
@@ -3181,7 +3195,7 @@
       <c r="L45" s="8"/>
       <c r="M45" s="2"/>
     </row>
-    <row r="46" spans="1:13">
+    <row r="46" spans="1:13" hidden="1">
       <c r="A46" s="8" t="s">
         <v>186</v>
       </c>
@@ -3214,7 +3228,7 @@
       <c r="L46" s="8"/>
       <c r="M46" s="2"/>
     </row>
-    <row r="47" spans="1:13">
+    <row r="47" spans="1:13" hidden="1">
       <c r="A47" s="8" t="s">
         <v>186</v>
       </c>
@@ -3247,7 +3261,7 @@
       <c r="L47" s="8"/>
       <c r="M47" s="2"/>
     </row>
-    <row r="48" spans="1:13">
+    <row r="48" spans="1:13" hidden="1">
       <c r="A48" s="8" t="s">
         <v>186</v>
       </c>
@@ -3280,7 +3294,7 @@
       <c r="L48" s="8"/>
       <c r="M48" s="2"/>
     </row>
-    <row r="49" spans="1:13">
+    <row r="49" spans="1:13" hidden="1">
       <c r="A49" s="8" t="s">
         <v>186</v>
       </c>
@@ -3313,7 +3327,7 @@
       <c r="L49" s="8"/>
       <c r="M49" s="2"/>
     </row>
-    <row r="50" spans="1:13">
+    <row r="50" spans="1:13" hidden="1">
       <c r="A50" s="8" t="s">
         <v>186</v>
       </c>
@@ -3346,7 +3360,7 @@
       <c r="L50" s="8"/>
       <c r="M50" s="2"/>
     </row>
-    <row r="51" spans="1:13">
+    <row r="51" spans="1:13" hidden="1">
       <c r="A51" s="8" t="s">
         <v>199</v>
       </c>
@@ -3379,7 +3393,7 @@
       <c r="L51" s="8"/>
       <c r="M51" s="2"/>
     </row>
-    <row r="52" spans="1:13">
+    <row r="52" spans="1:13" hidden="1">
       <c r="A52" s="8" t="s">
         <v>204</v>
       </c>
@@ -3412,7 +3426,7 @@
       <c r="L52" s="8"/>
       <c r="M52" s="2"/>
     </row>
-    <row r="53" spans="1:13">
+    <row r="53" spans="1:13" hidden="1">
       <c r="A53" s="8" t="s">
         <v>208</v>
       </c>
@@ -3445,7 +3459,7 @@
       <c r="L53" s="8"/>
       <c r="M53" s="2"/>
     </row>
-    <row r="54" spans="1:13">
+    <row r="54" spans="1:13" hidden="1">
       <c r="A54" s="8" t="s">
         <v>208</v>
       </c>
@@ -3478,7 +3492,7 @@
       <c r="L54" s="8"/>
       <c r="M54" s="2"/>
     </row>
-    <row r="55" spans="1:13">
+    <row r="55" spans="1:13" hidden="1">
       <c r="A55" s="8" t="s">
         <v>208</v>
       </c>
@@ -3511,7 +3525,7 @@
       <c r="L55" s="8"/>
       <c r="M55" s="2"/>
     </row>
-    <row r="56" spans="1:13">
+    <row r="56" spans="1:13" hidden="1">
       <c r="A56" s="8" t="s">
         <v>208</v>
       </c>
@@ -3620,7 +3634,14 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L57" xr:uid="{00000000-0001-0000-0200-000000000000}"/>
+  <autoFilter ref="A1:L57" xr:uid="{00000000-0001-0000-0200-000000000000}">
+    <filterColumn colId="6">
+      <filters>
+        <filter val="Blocked"/>
+        <filter val="Not Started"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G58:G115" xr:uid="{1210C842-B0BE-400E-882F-F7207D6FFCF0}">
       <formula1>INDIRECT("Status")</formula1>

</xml_diff>

<commit_message>
- Conditionally rendering driver coordination hint - DONE
- Animate pulse ongoing trip labels to make it visually feel that trip is live - DONE

- If upgradation information from server is not available(for some reason) by function getUpgradeMessage - then as a fallback -  try to make a upgrade message if possible by checking the trips' preferred car and fuel and the assigned drivers' car and fuel. DONE
</commit_message>
<xml_diff>
--- a/docs/customer-frontend-qa-checklist-local-env.xlsx
+++ b/docs/customer-frontend-qa-checklist-local-env.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ayanc\OneDrive\Desktop\cabbo-frontends\cabbo-customer-frontend\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{047868DB-7C4B-40C1-9A9C-CD0EC7A5409E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBCE4B94-B6EB-4002-B9E1-BDFC53B74575}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="559" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="562" uniqueCount="264">
   <si>
     <t>Generated for local QA run</t>
   </si>
@@ -837,7 +837,13 @@
     <t>Customer B (Oyendrila)</t>
   </si>
   <si>
-    <t>Will do once I complete admin panel - so I can enough data to perform this step</t>
+    <t>BUG-008</t>
+  </si>
+  <si>
+    <t>16th August 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">On opening a completed trip of any type and providing a review updates the DB and also UI reflects the changes locally from state data - but go back and again come here - it still shows - Provide review and not the recently provided review. Only after a page refresh the issue gets resolved - perhaps a react query state update issue. </t>
   </si>
 </sst>
 </file>
@@ -1508,7 +1514,7 @@
       </c>
       <c r="B4" s="13">
         <f>COUNTIF(Checklist!G2:G200,"Success")</f>
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="C4" s="2"/>
     </row>
@@ -1528,7 +1534,7 @@
       </c>
       <c r="B6" s="13">
         <f>COUNTIF(Checklist!G2:G200,"Blocked")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C6" s="2"/>
     </row>
@@ -1538,7 +1544,7 @@
       </c>
       <c r="B7" s="13">
         <f>COUNTIF(Checklist!G2:G200,"Not Started")</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="C7" s="2"/>
     </row>
@@ -1686,7 +1692,6 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:M75"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
@@ -1743,7 +1748,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:13" hidden="1">
+    <row r="2" spans="1:13">
       <c r="A2" s="8" t="s">
         <v>33</v>
       </c>
@@ -1776,7 +1781,7 @@
       <c r="L2" s="8"/>
       <c r="M2" s="2"/>
     </row>
-    <row r="3" spans="1:13" hidden="1">
+    <row r="3" spans="1:13">
       <c r="A3" s="8" t="s">
         <v>33</v>
       </c>
@@ -1809,7 +1814,7 @@
       <c r="L3" s="8"/>
       <c r="M3" s="2"/>
     </row>
-    <row r="4" spans="1:13" hidden="1">
+    <row r="4" spans="1:13">
       <c r="A4" s="8" t="s">
         <v>43</v>
       </c>
@@ -1842,7 +1847,7 @@
       <c r="L4" s="8"/>
       <c r="M4" s="2"/>
     </row>
-    <row r="5" spans="1:13" hidden="1">
+    <row r="5" spans="1:13">
       <c r="A5" s="8" t="s">
         <v>43</v>
       </c>
@@ -1875,7 +1880,7 @@
       <c r="L5" s="8"/>
       <c r="M5" s="2"/>
     </row>
-    <row r="6" spans="1:13" hidden="1">
+    <row r="6" spans="1:13">
       <c r="A6" s="8" t="s">
         <v>43</v>
       </c>
@@ -1908,7 +1913,7 @@
       <c r="L6" s="8"/>
       <c r="M6" s="2"/>
     </row>
-    <row r="7" spans="1:13" hidden="1">
+    <row r="7" spans="1:13">
       <c r="A7" s="8" t="s">
         <v>43</v>
       </c>
@@ -1941,7 +1946,7 @@
       <c r="L7" s="8"/>
       <c r="M7" s="2"/>
     </row>
-    <row r="8" spans="1:13" hidden="1">
+    <row r="8" spans="1:13">
       <c r="A8" s="8" t="s">
         <v>43</v>
       </c>
@@ -1974,7 +1979,7 @@
       <c r="L8" s="8"/>
       <c r="M8" s="2"/>
     </row>
-    <row r="9" spans="1:13" hidden="1">
+    <row r="9" spans="1:13">
       <c r="A9" s="8" t="s">
         <v>43</v>
       </c>
@@ -2007,7 +2012,7 @@
       <c r="L9" s="8"/>
       <c r="M9" s="2"/>
     </row>
-    <row r="10" spans="1:13" hidden="1">
+    <row r="10" spans="1:13">
       <c r="A10" s="8" t="s">
         <v>43</v>
       </c>
@@ -2040,7 +2045,7 @@
       <c r="L10" s="8"/>
       <c r="M10" s="2"/>
     </row>
-    <row r="11" spans="1:13" hidden="1">
+    <row r="11" spans="1:13">
       <c r="A11" s="8" t="s">
         <v>43</v>
       </c>
@@ -2073,7 +2078,7 @@
       <c r="L11" s="8"/>
       <c r="M11" s="2"/>
     </row>
-    <row r="12" spans="1:13" hidden="1">
+    <row r="12" spans="1:13">
       <c r="A12" s="8" t="s">
         <v>43</v>
       </c>
@@ -2106,7 +2111,7 @@
       <c r="L12" s="8"/>
       <c r="M12" s="2"/>
     </row>
-    <row r="13" spans="1:13" hidden="1">
+    <row r="13" spans="1:13">
       <c r="A13" s="8" t="s">
         <v>71</v>
       </c>
@@ -2139,7 +2144,7 @@
       <c r="L13" s="8"/>
       <c r="M13" s="2"/>
     </row>
-    <row r="14" spans="1:13" hidden="1">
+    <row r="14" spans="1:13">
       <c r="A14" s="8" t="s">
         <v>71</v>
       </c>
@@ -2172,7 +2177,7 @@
       <c r="L14" s="8"/>
       <c r="M14" s="2"/>
     </row>
-    <row r="15" spans="1:13" hidden="1">
+    <row r="15" spans="1:13">
       <c r="A15" s="8" t="s">
         <v>78</v>
       </c>
@@ -2205,7 +2210,7 @@
       <c r="L15" s="8"/>
       <c r="M15" s="2"/>
     </row>
-    <row r="16" spans="1:13" hidden="1">
+    <row r="16" spans="1:13">
       <c r="A16" s="8" t="s">
         <v>78</v>
       </c>
@@ -2238,7 +2243,7 @@
       <c r="L16" s="8"/>
       <c r="M16" s="2"/>
     </row>
-    <row r="17" spans="1:13" hidden="1">
+    <row r="17" spans="1:13">
       <c r="A17" s="8" t="s">
         <v>78</v>
       </c>
@@ -2271,7 +2276,7 @@
       <c r="L17" s="8"/>
       <c r="M17" s="2"/>
     </row>
-    <row r="18" spans="1:13" hidden="1">
+    <row r="18" spans="1:13">
       <c r="A18" s="8" t="s">
         <v>88</v>
       </c>
@@ -2304,7 +2309,7 @@
       <c r="L18" s="8"/>
       <c r="M18" s="2"/>
     </row>
-    <row r="19" spans="1:13" hidden="1">
+    <row r="19" spans="1:13">
       <c r="A19" s="8" t="s">
         <v>88</v>
       </c>
@@ -2337,7 +2342,7 @@
       <c r="L19" s="8"/>
       <c r="M19" s="2"/>
     </row>
-    <row r="20" spans="1:13" hidden="1">
+    <row r="20" spans="1:13">
       <c r="A20" s="8" t="s">
         <v>88</v>
       </c>
@@ -2370,7 +2375,7 @@
       <c r="L20" s="8"/>
       <c r="M20" s="2"/>
     </row>
-    <row r="21" spans="1:13" hidden="1">
+    <row r="21" spans="1:13">
       <c r="A21" s="8" t="s">
         <v>88</v>
       </c>
@@ -2403,7 +2408,7 @@
       <c r="L21" s="8"/>
       <c r="M21" s="2"/>
     </row>
-    <row r="22" spans="1:13" hidden="1">
+    <row r="22" spans="1:13">
       <c r="A22" s="8" t="s">
         <v>88</v>
       </c>
@@ -2436,7 +2441,7 @@
       <c r="L22" s="8"/>
       <c r="M22" s="2"/>
     </row>
-    <row r="23" spans="1:13" hidden="1">
+    <row r="23" spans="1:13">
       <c r="A23" s="8" t="s">
         <v>104</v>
       </c>
@@ -2469,7 +2474,7 @@
       <c r="L23" s="8"/>
       <c r="M23" s="2"/>
     </row>
-    <row r="24" spans="1:13" hidden="1">
+    <row r="24" spans="1:13">
       <c r="A24" s="8" t="s">
         <v>104</v>
       </c>
@@ -2502,7 +2507,7 @@
       <c r="L24" s="10"/>
       <c r="M24" s="2"/>
     </row>
-    <row r="25" spans="1:13" hidden="1">
+    <row r="25" spans="1:13">
       <c r="A25" s="8" t="s">
         <v>111</v>
       </c>
@@ -2535,7 +2540,7 @@
       <c r="L25" s="8"/>
       <c r="M25" s="2"/>
     </row>
-    <row r="26" spans="1:13" hidden="1">
+    <row r="26" spans="1:13">
       <c r="A26" s="8" t="s">
         <v>111</v>
       </c>
@@ -2568,7 +2573,7 @@
       <c r="L26" s="8"/>
       <c r="M26" s="2"/>
     </row>
-    <row r="27" spans="1:13" hidden="1">
+    <row r="27" spans="1:13">
       <c r="A27" s="8" t="s">
         <v>111</v>
       </c>
@@ -2601,7 +2606,7 @@
       <c r="L27" s="8"/>
       <c r="M27" s="2"/>
     </row>
-    <row r="28" spans="1:13" hidden="1">
+    <row r="28" spans="1:13">
       <c r="A28" s="8" t="s">
         <v>121</v>
       </c>
@@ -2653,18 +2658,18 @@
       <c r="F29" s="8" t="s">
         <v>128</v>
       </c>
-      <c r="G29" s="8" t="s">
-        <v>39</v>
+      <c r="G29" s="15" t="s">
+        <v>230</v>
       </c>
       <c r="H29" s="8" t="s">
         <v>228</v>
       </c>
-      <c r="I29" s="9"/>
+      <c r="I29" s="9">
+        <v>46250</v>
+      </c>
       <c r="J29" s="8"/>
       <c r="K29" s="8"/>
-      <c r="L29" s="8" t="s">
-        <v>261</v>
-      </c>
+      <c r="L29" s="8"/>
       <c r="M29" s="2"/>
     </row>
     <row r="30" spans="1:13">
@@ -2686,21 +2691,21 @@
       <c r="F30" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="G30" s="8" t="s">
-        <v>39</v>
+      <c r="G30" s="15" t="s">
+        <v>230</v>
       </c>
       <c r="H30" s="8" t="s">
         <v>228</v>
       </c>
-      <c r="I30" s="9"/>
+      <c r="I30" s="9">
+        <v>46250</v>
+      </c>
       <c r="J30" s="8"/>
       <c r="K30" s="8"/>
-      <c r="L30" s="8" t="s">
-        <v>261</v>
-      </c>
+      <c r="L30" s="8"/>
       <c r="M30" s="2"/>
     </row>
-    <row r="31" spans="1:13" hidden="1">
+    <row r="31" spans="1:13">
       <c r="A31" s="8" t="s">
         <v>121</v>
       </c>
@@ -2752,18 +2757,18 @@
       <c r="F32" s="8" t="s">
         <v>137</v>
       </c>
-      <c r="G32" s="8" t="s">
-        <v>39</v>
+      <c r="G32" s="15" t="s">
+        <v>230</v>
       </c>
       <c r="H32" s="8" t="s">
         <v>228</v>
       </c>
-      <c r="I32" s="8"/>
+      <c r="I32" s="9">
+        <v>46250</v>
+      </c>
       <c r="J32" s="8"/>
       <c r="K32" s="8"/>
-      <c r="L32" s="8" t="s">
-        <v>261</v>
-      </c>
+      <c r="L32" s="8"/>
       <c r="M32" s="2"/>
     </row>
     <row r="33" spans="1:13">
@@ -2785,18 +2790,18 @@
       <c r="F33" s="8" t="s">
         <v>140</v>
       </c>
-      <c r="G33" s="8" t="s">
-        <v>39</v>
+      <c r="G33" s="15" t="s">
+        <v>230</v>
       </c>
       <c r="H33" s="8" t="s">
         <v>228</v>
       </c>
-      <c r="I33" s="8"/>
+      <c r="I33" s="9">
+        <v>46250</v>
+      </c>
       <c r="J33" s="8"/>
       <c r="K33" s="8"/>
-      <c r="L33" s="8" t="s">
-        <v>261</v>
-      </c>
+      <c r="L33" s="8"/>
       <c r="M33" s="2"/>
     </row>
     <row r="34" spans="1:13">
@@ -2818,21 +2823,21 @@
       <c r="F34" s="8" t="s">
         <v>144</v>
       </c>
-      <c r="G34" s="8" t="s">
-        <v>39</v>
+      <c r="G34" s="15" t="s">
+        <v>230</v>
       </c>
       <c r="H34" s="8" t="s">
         <v>228</v>
       </c>
-      <c r="I34" s="8"/>
+      <c r="I34" s="9">
+        <v>46250</v>
+      </c>
       <c r="J34" s="8"/>
       <c r="K34" s="8"/>
-      <c r="L34" s="8" t="s">
-        <v>261</v>
-      </c>
+      <c r="L34" s="8"/>
       <c r="M34" s="2"/>
     </row>
-    <row r="35" spans="1:13" hidden="1">
+    <row r="35" spans="1:13">
       <c r="A35" s="8" t="s">
         <v>141</v>
       </c>
@@ -2865,7 +2870,7 @@
       <c r="L35" s="8"/>
       <c r="M35" s="2"/>
     </row>
-    <row r="36" spans="1:13" hidden="1">
+    <row r="36" spans="1:13">
       <c r="A36" s="8" t="s">
         <v>147</v>
       </c>
@@ -2898,7 +2903,7 @@
       <c r="L36" s="8"/>
       <c r="M36" s="2"/>
     </row>
-    <row r="37" spans="1:13" hidden="1">
+    <row r="37" spans="1:13">
       <c r="A37" s="8" t="s">
         <v>147</v>
       </c>
@@ -2931,7 +2936,7 @@
       <c r="L37" s="8"/>
       <c r="M37" s="2"/>
     </row>
-    <row r="38" spans="1:13" hidden="1">
+    <row r="38" spans="1:13">
       <c r="A38" s="8" t="s">
         <v>147</v>
       </c>
@@ -2964,7 +2969,7 @@
       <c r="L38" s="8"/>
       <c r="M38" s="2"/>
     </row>
-    <row r="39" spans="1:13" hidden="1">
+    <row r="39" spans="1:13">
       <c r="A39" s="8" t="s">
         <v>158</v>
       </c>
@@ -2997,7 +3002,7 @@
       <c r="L39" s="8"/>
       <c r="M39" s="2"/>
     </row>
-    <row r="40" spans="1:13" hidden="1">
+    <row r="40" spans="1:13">
       <c r="A40" s="8" t="s">
         <v>158</v>
       </c>
@@ -3030,7 +3035,7 @@
       <c r="L40" s="8"/>
       <c r="M40" s="2"/>
     </row>
-    <row r="41" spans="1:13" hidden="1">
+    <row r="41" spans="1:13">
       <c r="A41" s="8" t="s">
         <v>166</v>
       </c>
@@ -3063,7 +3068,7 @@
       <c r="L41" s="8"/>
       <c r="M41" s="2"/>
     </row>
-    <row r="42" spans="1:13" hidden="1">
+    <row r="42" spans="1:13">
       <c r="A42" s="8" t="s">
         <v>166</v>
       </c>
@@ -3096,7 +3101,7 @@
       <c r="L42" s="8"/>
       <c r="M42" s="2"/>
     </row>
-    <row r="43" spans="1:13" hidden="1">
+    <row r="43" spans="1:13">
       <c r="A43" s="8" t="s">
         <v>166</v>
       </c>
@@ -3129,7 +3134,7 @@
       <c r="L43" s="8"/>
       <c r="M43" s="2"/>
     </row>
-    <row r="44" spans="1:13" hidden="1">
+    <row r="44" spans="1:13">
       <c r="A44" s="8" t="s">
         <v>166</v>
       </c>
@@ -3162,7 +3167,7 @@
       <c r="L44" s="8"/>
       <c r="M44" s="2"/>
     </row>
-    <row r="45" spans="1:13" hidden="1">
+    <row r="45" spans="1:13">
       <c r="A45" s="8" t="s">
         <v>166</v>
       </c>
@@ -3195,7 +3200,7 @@
       <c r="L45" s="8"/>
       <c r="M45" s="2"/>
     </row>
-    <row r="46" spans="1:13" hidden="1">
+    <row r="46" spans="1:13">
       <c r="A46" s="8" t="s">
         <v>186</v>
       </c>
@@ -3228,7 +3233,7 @@
       <c r="L46" s="8"/>
       <c r="M46" s="2"/>
     </row>
-    <row r="47" spans="1:13" hidden="1">
+    <row r="47" spans="1:13">
       <c r="A47" s="8" t="s">
         <v>186</v>
       </c>
@@ -3261,7 +3266,7 @@
       <c r="L47" s="8"/>
       <c r="M47" s="2"/>
     </row>
-    <row r="48" spans="1:13" hidden="1">
+    <row r="48" spans="1:13">
       <c r="A48" s="8" t="s">
         <v>186</v>
       </c>
@@ -3294,7 +3299,7 @@
       <c r="L48" s="8"/>
       <c r="M48" s="2"/>
     </row>
-    <row r="49" spans="1:13" hidden="1">
+    <row r="49" spans="1:13">
       <c r="A49" s="8" t="s">
         <v>186</v>
       </c>
@@ -3327,7 +3332,7 @@
       <c r="L49" s="8"/>
       <c r="M49" s="2"/>
     </row>
-    <row r="50" spans="1:13" hidden="1">
+    <row r="50" spans="1:13">
       <c r="A50" s="8" t="s">
         <v>186</v>
       </c>
@@ -3360,7 +3365,7 @@
       <c r="L50" s="8"/>
       <c r="M50" s="2"/>
     </row>
-    <row r="51" spans="1:13" hidden="1">
+    <row r="51" spans="1:13">
       <c r="A51" s="8" t="s">
         <v>199</v>
       </c>
@@ -3393,7 +3398,7 @@
       <c r="L51" s="8"/>
       <c r="M51" s="2"/>
     </row>
-    <row r="52" spans="1:13" hidden="1">
+    <row r="52" spans="1:13">
       <c r="A52" s="8" t="s">
         <v>204</v>
       </c>
@@ -3426,7 +3431,7 @@
       <c r="L52" s="8"/>
       <c r="M52" s="2"/>
     </row>
-    <row r="53" spans="1:13" hidden="1">
+    <row r="53" spans="1:13">
       <c r="A53" s="8" t="s">
         <v>208</v>
       </c>
@@ -3459,7 +3464,7 @@
       <c r="L53" s="8"/>
       <c r="M53" s="2"/>
     </row>
-    <row r="54" spans="1:13" hidden="1">
+    <row r="54" spans="1:13">
       <c r="A54" s="8" t="s">
         <v>208</v>
       </c>
@@ -3492,7 +3497,7 @@
       <c r="L54" s="8"/>
       <c r="M54" s="2"/>
     </row>
-    <row r="55" spans="1:13" hidden="1">
+    <row r="55" spans="1:13">
       <c r="A55" s="8" t="s">
         <v>208</v>
       </c>
@@ -3525,7 +3530,7 @@
       <c r="L55" s="8"/>
       <c r="M55" s="2"/>
     </row>
-    <row r="56" spans="1:13" hidden="1">
+    <row r="56" spans="1:13">
       <c r="A56" s="8" t="s">
         <v>208</v>
       </c>
@@ -3577,13 +3582,15 @@
       <c r="F57" s="8" t="s">
         <v>218</v>
       </c>
-      <c r="G57" s="8" t="s">
-        <v>4</v>
+      <c r="G57" s="15" t="s">
+        <v>230</v>
       </c>
       <c r="H57" s="8" t="s">
         <v>228</v>
       </c>
-      <c r="I57" s="8"/>
+      <c r="I57" s="9">
+        <v>46250</v>
+      </c>
       <c r="J57" s="8"/>
       <c r="K57" s="8"/>
       <c r="L57" s="8"/>
@@ -3634,14 +3641,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L57" xr:uid="{00000000-0001-0000-0200-000000000000}">
-    <filterColumn colId="6">
-      <filters>
-        <filter val="Blocked"/>
-        <filter val="Not Started"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:L57" xr:uid="{00000000-0001-0000-0200-000000000000}"/>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G58:G115" xr:uid="{1210C842-B0BE-400E-882F-F7207D6FFCF0}">
       <formula1>INDIRECT("Status")</formula1>
@@ -3659,7 +3659,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
@@ -3886,15 +3886,164 @@
       </c>
       <c r="I8" s="22"/>
     </row>
-    <row r="9" spans="1:9">
-      <c r="A9" s="6"/>
-      <c r="B9" s="6"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
-      <c r="H9" s="6"/>
+    <row r="9" spans="1:9" ht="119" customHeight="1">
+      <c r="A9" s="20" t="s">
+        <v>261</v>
+      </c>
+      <c r="B9" s="20" t="s">
+        <v>262</v>
+      </c>
+      <c r="C9" s="20" t="s">
+        <v>122</v>
+      </c>
+      <c r="D9" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="E9" s="20" t="s">
+        <v>240</v>
+      </c>
+      <c r="F9" s="20" t="s">
+        <v>258</v>
+      </c>
+      <c r="G9" s="20" t="s">
+        <v>228</v>
+      </c>
+      <c r="H9" s="20" t="s">
+        <v>263</v>
+      </c>
+      <c r="I9" s="2"/>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" s="8"/>
+      <c r="B10" s="8"/>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="2"/>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" s="8"/>
+      <c r="B11" s="8"/>
+      <c r="C11" s="8"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="2"/>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" s="8"/>
+      <c r="B12" s="8"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="8"/>
+      <c r="I12" s="2"/>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" s="8"/>
+      <c r="B13" s="8"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
+      <c r="I13" s="2"/>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14" s="8"/>
+      <c r="B14" s="8"/>
+      <c r="C14" s="8"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="8"/>
+      <c r="I14" s="2"/>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="A15" s="8"/>
+      <c r="B15" s="8"/>
+      <c r="C15" s="8"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="8"/>
+      <c r="I15" s="2"/>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="A16" s="8"/>
+      <c r="B16" s="8"/>
+      <c r="C16" s="8"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="8"/>
+      <c r="H16" s="8"/>
+      <c r="I16" s="2"/>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" s="8"/>
+      <c r="B17" s="8"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8"/>
+      <c r="I17" s="2"/>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18" s="8"/>
+      <c r="B18" s="8"/>
+      <c r="C18" s="8"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
+      <c r="G18" s="8"/>
+      <c r="H18" s="8"/>
+      <c r="I18" s="2"/>
+    </row>
+    <row r="19" spans="1:9">
+      <c r="A19" s="8"/>
+      <c r="B19" s="8"/>
+      <c r="C19" s="8"/>
+      <c r="D19" s="8"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="8"/>
+      <c r="G19" s="8"/>
+      <c r="H19" s="8"/>
+      <c r="I19" s="2"/>
+    </row>
+    <row r="20" spans="1:9">
+      <c r="A20" s="8"/>
+      <c r="B20" s="8"/>
+      <c r="C20" s="8"/>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="8"/>
+      <c r="G20" s="8"/>
+      <c r="H20" s="8"/>
+      <c r="I20" s="2"/>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="A21" s="8"/>
+      <c r="B21" s="8"/>
+      <c r="C21" s="8"/>
+      <c r="D21" s="8"/>
+      <c r="E21" s="8"/>
+      <c r="F21" s="8"/>
+      <c r="G21" s="8"/>
+      <c r="H21" s="8"/>
+      <c r="I21" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>